<commit_message>
Added Exercise 4B excel
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_GTrends.xlsx
+++ b/week-01/Ex4A_GTrends.xlsx
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">GTrends_milkshake_hamburger_202!$A$1:$E$52</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>